<commit_message>
Ajout des structure Transform et Collider
- Ajout de la structure Transform
- Ajout du singleton Graphics
- Ajout de la structure Math
- Ajout de la structure Collider avec :
   - L'algorithme de Gilbert–Johnson–Keerthi
   - Le support Minkowski
</commit_message>
<xml_diff>
--- a/Matrice des tâches.xlsx
+++ b/Matrice des tâches.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="20">
   <si>
     <t xml:space="preserve">Matrice de répartition de charges (à remplir à chaque séance)</t>
   </si>
@@ -53,6 +53,9 @@
   </si>
   <si>
     <t xml:space="preserve">Création du GitHub</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ajout de la structure transform et de la structure collider avec l’algorithme de Gilbert–Johnson–Keerthi et le supportMinkowski </t>
   </si>
   <si>
     <t xml:space="preserve">Attention :</t>
@@ -291,7 +294,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="22">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -304,7 +307,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -320,7 +323,7 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="7" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -328,7 +331,7 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="2" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="2" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -336,23 +339,15 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="2" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="3" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="3" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -466,15 +461,15 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:H29"/>
-  <sheetFormatPr defaultColWidth="8.6875" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6953125" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="9.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14.87"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="9.13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14.88"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="22.23"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="19.08"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="35.15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="23.06"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="7" style="0" width="9.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="23.07"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="7" style="0" width="9.13"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -570,112 +565,120 @@
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1"/>
-      <c r="B8" s="8"/>
-      <c r="C8" s="11"/>
-      <c r="D8" s="11"/>
-      <c r="E8" s="11"/>
-      <c r="F8" s="11"/>
+      <c r="B8" s="7" t="n">
+        <v>46275</v>
+      </c>
+      <c r="C8" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D8" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="E8" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="F8" s="8"/>
       <c r="G8" s="1"/>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1"/>
-      <c r="B9" s="6"/>
-      <c r="C9" s="12"/>
-      <c r="D9" s="12"/>
-      <c r="E9" s="12"/>
-      <c r="F9" s="12"/>
+      <c r="B9" s="10"/>
+      <c r="C9" s="10"/>
+      <c r="D9" s="10"/>
+      <c r="E9" s="10"/>
+      <c r="F9" s="10"/>
       <c r="G9" s="1"/>
-      <c r="H9" s="13"/>
+      <c r="H9" s="11"/>
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1"/>
       <c r="B10" s="8"/>
       <c r="C10" s="8"/>
-      <c r="D10" s="11"/>
+      <c r="D10" s="8"/>
       <c r="E10" s="8"/>
       <c r="F10" s="8"/>
       <c r="G10" s="1"/>
-      <c r="H10" s="13"/>
+      <c r="H10" s="11"/>
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1"/>
-      <c r="B11" s="14"/>
-      <c r="C11" s="14"/>
-      <c r="D11" s="14"/>
-      <c r="E11" s="14"/>
-      <c r="F11" s="14"/>
+      <c r="B11" s="12"/>
+      <c r="C11" s="12"/>
+      <c r="D11" s="12"/>
+      <c r="E11" s="12"/>
+      <c r="F11" s="12"/>
       <c r="G11" s="1"/>
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1"/>
-      <c r="B12" s="15"/>
-      <c r="C12" s="15"/>
-      <c r="D12" s="15"/>
-      <c r="E12" s="15"/>
-      <c r="F12" s="15"/>
+      <c r="B12" s="13"/>
+      <c r="C12" s="13"/>
+      <c r="D12" s="13"/>
+      <c r="E12" s="13"/>
+      <c r="F12" s="13"/>
       <c r="G12" s="1"/>
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1"/>
-      <c r="B13" s="14"/>
-      <c r="C13" s="14"/>
-      <c r="D13" s="14"/>
-      <c r="E13" s="14"/>
-      <c r="F13" s="14"/>
+      <c r="B13" s="12"/>
+      <c r="C13" s="12"/>
+      <c r="D13" s="12"/>
+      <c r="E13" s="12"/>
+      <c r="F13" s="12"/>
       <c r="G13" s="1"/>
     </row>
     <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1"/>
-      <c r="B14" s="15"/>
-      <c r="C14" s="15"/>
-      <c r="D14" s="15"/>
-      <c r="E14" s="15"/>
-      <c r="F14" s="15"/>
+      <c r="B14" s="13"/>
+      <c r="C14" s="13"/>
+      <c r="D14" s="13"/>
+      <c r="E14" s="13"/>
+      <c r="F14" s="13"/>
       <c r="G14" s="1"/>
     </row>
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1"/>
-      <c r="B15" s="14"/>
-      <c r="C15" s="14"/>
-      <c r="D15" s="14"/>
-      <c r="E15" s="14"/>
-      <c r="F15" s="14"/>
+      <c r="B15" s="12"/>
+      <c r="C15" s="12"/>
+      <c r="D15" s="12"/>
+      <c r="E15" s="12"/>
+      <c r="F15" s="12"/>
       <c r="G15" s="1"/>
     </row>
     <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1"/>
-      <c r="B16" s="15"/>
-      <c r="C16" s="15"/>
-      <c r="D16" s="15"/>
-      <c r="E16" s="15"/>
-      <c r="F16" s="15"/>
+      <c r="B16" s="13"/>
+      <c r="C16" s="13"/>
+      <c r="D16" s="13"/>
+      <c r="E16" s="13"/>
+      <c r="F16" s="13"/>
       <c r="G16" s="1"/>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1"/>
-      <c r="B17" s="14"/>
-      <c r="C17" s="14"/>
-      <c r="D17" s="14"/>
-      <c r="E17" s="14"/>
-      <c r="F17" s="14"/>
+      <c r="B17" s="12"/>
+      <c r="C17" s="12"/>
+      <c r="D17" s="12"/>
+      <c r="E17" s="12"/>
+      <c r="F17" s="12"/>
       <c r="G17" s="1"/>
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1"/>
-      <c r="B18" s="15"/>
-      <c r="C18" s="15"/>
-      <c r="D18" s="15"/>
-      <c r="E18" s="15"/>
-      <c r="F18" s="15"/>
+      <c r="B18" s="13"/>
+      <c r="C18" s="13"/>
+      <c r="D18" s="13"/>
+      <c r="E18" s="13"/>
+      <c r="F18" s="13"/>
       <c r="G18" s="1"/>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1"/>
-      <c r="B19" s="14"/>
-      <c r="C19" s="14"/>
-      <c r="D19" s="14"/>
-      <c r="E19" s="14"/>
-      <c r="F19" s="14"/>
+      <c r="B19" s="12"/>
+      <c r="C19" s="12"/>
+      <c r="D19" s="12"/>
+      <c r="E19" s="12"/>
+      <c r="F19" s="12"/>
       <c r="G19" s="1"/>
     </row>
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -689,92 +692,92 @@
     </row>
     <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1"/>
-      <c r="B21" s="16" t="s">
-        <v>11</v>
-      </c>
-      <c r="C21" s="17"/>
-      <c r="D21" s="17"/>
-      <c r="E21" s="17"/>
-      <c r="F21" s="18"/>
+      <c r="B21" s="14" t="s">
+        <v>12</v>
+      </c>
+      <c r="C21" s="15"/>
+      <c r="D21" s="15"/>
+      <c r="E21" s="15"/>
+      <c r="F21" s="16"/>
       <c r="G21" s="1"/>
     </row>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1"/>
-      <c r="B22" s="19"/>
+      <c r="B22" s="17"/>
       <c r="C22" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D22" s="1"/>
       <c r="E22" s="1"/>
-      <c r="F22" s="20"/>
+      <c r="F22" s="18"/>
       <c r="G22" s="1"/>
     </row>
     <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="1"/>
-      <c r="B23" s="19"/>
+      <c r="B23" s="17"/>
       <c r="C23" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D23" s="1"/>
       <c r="E23" s="1"/>
-      <c r="F23" s="20"/>
+      <c r="F23" s="18"/>
       <c r="G23" s="1"/>
-      <c r="H23" s="13"/>
+      <c r="H23" s="11"/>
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="1"/>
-      <c r="B24" s="19"/>
+      <c r="B24" s="17"/>
       <c r="C24" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D24" s="1"/>
       <c r="E24" s="1"/>
-      <c r="F24" s="20"/>
+      <c r="F24" s="18"/>
       <c r="G24" s="1"/>
-      <c r="H24" s="13"/>
+      <c r="H24" s="11"/>
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="1"/>
-      <c r="B25" s="19"/>
+      <c r="B25" s="17"/>
       <c r="C25" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D25" s="1"/>
       <c r="E25" s="1"/>
-      <c r="F25" s="20"/>
+      <c r="F25" s="18"/>
       <c r="G25" s="1"/>
     </row>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="1"/>
-      <c r="B26" s="19"/>
+      <c r="B26" s="17"/>
       <c r="C26" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D26" s="1"/>
       <c r="E26" s="1"/>
-      <c r="F26" s="20"/>
+      <c r="F26" s="18"/>
       <c r="G26" s="1"/>
     </row>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="1"/>
-      <c r="B27" s="19"/>
+      <c r="B27" s="17"/>
       <c r="C27" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D27" s="1"/>
       <c r="E27" s="1"/>
-      <c r="F27" s="20"/>
+      <c r="F27" s="18"/>
       <c r="G27" s="1"/>
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="1"/>
-      <c r="B28" s="21"/>
-      <c r="C28" s="22" t="s">
-        <v>18</v>
-      </c>
-      <c r="D28" s="22"/>
-      <c r="E28" s="22"/>
-      <c r="F28" s="23"/>
+      <c r="B28" s="19"/>
+      <c r="C28" s="20" t="s">
+        <v>19</v>
+      </c>
+      <c r="D28" s="20"/>
+      <c r="E28" s="20"/>
+      <c r="F28" s="21"/>
       <c r="G28" s="1"/>
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Ajout des tâches dans la matrice des tâches
- Ajout des tâches dans la matrice des tâches
</commit_message>
<xml_diff>
--- a/Matrice des tâches.xlsx
+++ b/Matrice des tâches.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="23">
   <si>
     <t xml:space="preserve">Matrice de répartition de charges (à remplir à chaque séance)</t>
   </si>
@@ -56,6 +56,15 @@
   </si>
   <si>
     <t xml:space="preserve">Ajout de la structure transform et de la structure collider avec l’algorithme de Gilbert–Johnson–Keerthi et le supportMinkowski </t>
+  </si>
+  <si>
+    <t xml:space="preserve">6h</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ajout des components Mareriel, PhysicsBody, et PhysicsWorld </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fait sur plusieurs cours</t>
   </si>
   <si>
     <t xml:space="preserve">Attention :</t>
@@ -294,7 +303,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -337,6 +346,10 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="2" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
@@ -461,14 +474,14 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:H29"/>
-  <sheetFormatPr defaultColWidth="8.6953125" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.70703125" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="9.13"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14.88"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="22.23"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="19.08"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="35.15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="23.07"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="23.08"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="7" style="0" width="9.13"/>
   </cols>
   <sheetData>
@@ -580,15 +593,25 @@
       <c r="F8" s="8"/>
       <c r="G8" s="1"/>
     </row>
-    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1"/>
-      <c r="B9" s="10"/>
-      <c r="C9" s="10"/>
-      <c r="D9" s="10"/>
-      <c r="E9" s="10"/>
-      <c r="F9" s="10"/>
+      <c r="B9" s="9" t="n">
+        <v>46282</v>
+      </c>
+      <c r="C9" s="10" t="s">
+        <v>6</v>
+      </c>
+      <c r="D9" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="E9" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F9" s="10" t="s">
+        <v>14</v>
+      </c>
       <c r="G9" s="1"/>
-      <c r="H9" s="11"/>
+      <c r="H9" s="12"/>
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1"/>
@@ -598,87 +621,87 @@
       <c r="E10" s="8"/>
       <c r="F10" s="8"/>
       <c r="G10" s="1"/>
-      <c r="H10" s="11"/>
+      <c r="H10" s="12"/>
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1"/>
-      <c r="B11" s="12"/>
-      <c r="C11" s="12"/>
-      <c r="D11" s="12"/>
-      <c r="E11" s="12"/>
-      <c r="F11" s="12"/>
+      <c r="B11" s="13"/>
+      <c r="C11" s="13"/>
+      <c r="D11" s="13"/>
+      <c r="E11" s="13"/>
+      <c r="F11" s="13"/>
       <c r="G11" s="1"/>
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1"/>
-      <c r="B12" s="13"/>
-      <c r="C12" s="13"/>
-      <c r="D12" s="13"/>
-      <c r="E12" s="13"/>
-      <c r="F12" s="13"/>
+      <c r="B12" s="14"/>
+      <c r="C12" s="14"/>
+      <c r="D12" s="14"/>
+      <c r="E12" s="14"/>
+      <c r="F12" s="14"/>
       <c r="G12" s="1"/>
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1"/>
-      <c r="B13" s="12"/>
-      <c r="C13" s="12"/>
-      <c r="D13" s="12"/>
-      <c r="E13" s="12"/>
-      <c r="F13" s="12"/>
+      <c r="B13" s="13"/>
+      <c r="C13" s="13"/>
+      <c r="D13" s="13"/>
+      <c r="E13" s="13"/>
+      <c r="F13" s="13"/>
       <c r="G13" s="1"/>
     </row>
     <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1"/>
-      <c r="B14" s="13"/>
-      <c r="C14" s="13"/>
-      <c r="D14" s="13"/>
-      <c r="E14" s="13"/>
-      <c r="F14" s="13"/>
+      <c r="B14" s="14"/>
+      <c r="C14" s="14"/>
+      <c r="D14" s="14"/>
+      <c r="E14" s="14"/>
+      <c r="F14" s="14"/>
       <c r="G14" s="1"/>
     </row>
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1"/>
-      <c r="B15" s="12"/>
-      <c r="C15" s="12"/>
-      <c r="D15" s="12"/>
-      <c r="E15" s="12"/>
-      <c r="F15" s="12"/>
+      <c r="B15" s="13"/>
+      <c r="C15" s="13"/>
+      <c r="D15" s="13"/>
+      <c r="E15" s="13"/>
+      <c r="F15" s="13"/>
       <c r="G15" s="1"/>
     </row>
     <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1"/>
-      <c r="B16" s="13"/>
-      <c r="C16" s="13"/>
-      <c r="D16" s="13"/>
-      <c r="E16" s="13"/>
-      <c r="F16" s="13"/>
+      <c r="B16" s="14"/>
+      <c r="C16" s="14"/>
+      <c r="D16" s="14"/>
+      <c r="E16" s="14"/>
+      <c r="F16" s="14"/>
       <c r="G16" s="1"/>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1"/>
-      <c r="B17" s="12"/>
-      <c r="C17" s="12"/>
-      <c r="D17" s="12"/>
-      <c r="E17" s="12"/>
-      <c r="F17" s="12"/>
+      <c r="B17" s="13"/>
+      <c r="C17" s="13"/>
+      <c r="D17" s="13"/>
+      <c r="E17" s="13"/>
+      <c r="F17" s="13"/>
       <c r="G17" s="1"/>
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1"/>
-      <c r="B18" s="13"/>
-      <c r="C18" s="13"/>
-      <c r="D18" s="13"/>
-      <c r="E18" s="13"/>
-      <c r="F18" s="13"/>
+      <c r="B18" s="14"/>
+      <c r="C18" s="14"/>
+      <c r="D18" s="14"/>
+      <c r="E18" s="14"/>
+      <c r="F18" s="14"/>
       <c r="G18" s="1"/>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1"/>
-      <c r="B19" s="12"/>
-      <c r="C19" s="12"/>
-      <c r="D19" s="12"/>
-      <c r="E19" s="12"/>
-      <c r="F19" s="12"/>
+      <c r="B19" s="13"/>
+      <c r="C19" s="13"/>
+      <c r="D19" s="13"/>
+      <c r="E19" s="13"/>
+      <c r="F19" s="13"/>
       <c r="G19" s="1"/>
     </row>
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -692,92 +715,92 @@
     </row>
     <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1"/>
-      <c r="B21" s="14" t="s">
-        <v>12</v>
-      </c>
-      <c r="C21" s="15"/>
-      <c r="D21" s="15"/>
-      <c r="E21" s="15"/>
-      <c r="F21" s="16"/>
+      <c r="B21" s="15" t="s">
+        <v>15</v>
+      </c>
+      <c r="C21" s="16"/>
+      <c r="D21" s="16"/>
+      <c r="E21" s="16"/>
+      <c r="F21" s="17"/>
       <c r="G21" s="1"/>
     </row>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1"/>
-      <c r="B22" s="17"/>
+      <c r="B22" s="18"/>
       <c r="C22" s="1" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="D22" s="1"/>
       <c r="E22" s="1"/>
-      <c r="F22" s="18"/>
+      <c r="F22" s="19"/>
       <c r="G22" s="1"/>
     </row>
     <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="1"/>
-      <c r="B23" s="17"/>
+      <c r="B23" s="18"/>
       <c r="C23" s="1" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D23" s="1"/>
       <c r="E23" s="1"/>
-      <c r="F23" s="18"/>
+      <c r="F23" s="19"/>
       <c r="G23" s="1"/>
-      <c r="H23" s="11"/>
+      <c r="H23" s="12"/>
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="1"/>
-      <c r="B24" s="17"/>
+      <c r="B24" s="18"/>
       <c r="C24" s="1" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="D24" s="1"/>
       <c r="E24" s="1"/>
-      <c r="F24" s="18"/>
+      <c r="F24" s="19"/>
       <c r="G24" s="1"/>
-      <c r="H24" s="11"/>
+      <c r="H24" s="12"/>
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="1"/>
-      <c r="B25" s="17"/>
+      <c r="B25" s="18"/>
       <c r="C25" s="1" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="D25" s="1"/>
       <c r="E25" s="1"/>
-      <c r="F25" s="18"/>
+      <c r="F25" s="19"/>
       <c r="G25" s="1"/>
     </row>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="1"/>
-      <c r="B26" s="17"/>
+      <c r="B26" s="18"/>
       <c r="C26" s="1" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="D26" s="1"/>
       <c r="E26" s="1"/>
-      <c r="F26" s="18"/>
+      <c r="F26" s="19"/>
       <c r="G26" s="1"/>
     </row>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="1"/>
-      <c r="B27" s="17"/>
+      <c r="B27" s="18"/>
       <c r="C27" s="1" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="D27" s="1"/>
       <c r="E27" s="1"/>
-      <c r="F27" s="18"/>
+      <c r="F27" s="19"/>
       <c r="G27" s="1"/>
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="1"/>
-      <c r="B28" s="19"/>
-      <c r="C28" s="20" t="s">
-        <v>19</v>
-      </c>
-      <c r="D28" s="20"/>
-      <c r="E28" s="20"/>
-      <c r="F28" s="21"/>
+      <c r="B28" s="20"/>
+      <c r="C28" s="21" t="s">
+        <v>22</v>
+      </c>
+      <c r="D28" s="21"/>
+      <c r="E28" s="21"/>
+      <c r="F28" s="22"/>
       <c r="G28" s="1"/>
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Ajout de la possibilité de changer la vitesse d'accélération et de décélération + Arrêt de l'entité
- Ajout de la possibilité de changer la vitesse d'accélération et de décélération
- Arrêt de l'entité
</commit_message>
<xml_diff>
--- a/Matrice des tâches.xlsx
+++ b/Matrice des tâches.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="24">
   <si>
     <t xml:space="preserve">Matrice de répartition de charges (à remplir à chaque séance)</t>
   </si>
@@ -65,6 +65,9 @@
   </si>
   <si>
     <t xml:space="preserve">Fait sur plusieurs cours</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ajout de la possibilité de changer la vitesse d'accélération et de décélération + Arrêt de l'entité</t>
   </si>
   <si>
     <t xml:space="preserve">Attention :</t>
@@ -474,7 +477,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:H29"/>
-  <sheetFormatPr defaultColWidth="8.70703125" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.72265625" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="9.13"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14.88"/>
@@ -615,10 +618,18 @@
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1"/>
-      <c r="B10" s="8"/>
-      <c r="C10" s="8"/>
-      <c r="D10" s="8"/>
-      <c r="E10" s="8"/>
+      <c r="B10" s="7" t="n">
+        <v>46287</v>
+      </c>
+      <c r="C10" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D10" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="E10" s="8" t="s">
+        <v>15</v>
+      </c>
       <c r="F10" s="8"/>
       <c r="G10" s="1"/>
       <c r="H10" s="12"/>
@@ -716,7 +727,7 @@
     <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1"/>
       <c r="B21" s="15" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C21" s="16"/>
       <c r="D21" s="16"/>
@@ -728,7 +739,7 @@
       <c r="A22" s="1"/>
       <c r="B22" s="18"/>
       <c r="C22" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D22" s="1"/>
       <c r="E22" s="1"/>
@@ -739,7 +750,7 @@
       <c r="A23" s="1"/>
       <c r="B23" s="18"/>
       <c r="C23" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D23" s="1"/>
       <c r="E23" s="1"/>
@@ -751,7 +762,7 @@
       <c r="A24" s="1"/>
       <c r="B24" s="18"/>
       <c r="C24" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D24" s="1"/>
       <c r="E24" s="1"/>
@@ -763,7 +774,7 @@
       <c r="A25" s="1"/>
       <c r="B25" s="18"/>
       <c r="C25" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D25" s="1"/>
       <c r="E25" s="1"/>
@@ -774,7 +785,7 @@
       <c r="A26" s="1"/>
       <c r="B26" s="18"/>
       <c r="C26" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D26" s="1"/>
       <c r="E26" s="1"/>
@@ -785,7 +796,7 @@
       <c r="A27" s="1"/>
       <c r="B27" s="18"/>
       <c r="C27" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D27" s="1"/>
       <c r="E27" s="1"/>
@@ -796,7 +807,7 @@
       <c r="A28" s="1"/>
       <c r="B28" s="20"/>
       <c r="C28" s="21" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D28" s="21"/>
       <c r="E28" s="21"/>

</xml_diff>

<commit_message>
Ajout du fichier glkresult
- Ajout du fichier glkresult
- Modification de nextSimplex pour revoyer true seulement avec trois simplexe ( pour EPA )
</commit_message>
<xml_diff>
--- a/Matrice des tâches.xlsx
+++ b/Matrice des tâches.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="26">
   <si>
     <t xml:space="preserve">Matrice de répartition de charges (à remplir à chaque séance)</t>
   </si>
@@ -68,6 +68,12 @@
   </si>
   <si>
     <t xml:space="preserve">Ajout de la possibilité de changer la vitesse d'accélération et de décélération + Arrêt de l'entité</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ajout du fichier glkresult</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J’ai aussi bien réfléchit sur comment implémenter les collisions entre entité</t>
   </si>
   <si>
     <t xml:space="preserve">Attention :</t>
@@ -306,7 +312,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="24">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -357,6 +363,10 @@
     </xf>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="2" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="2" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
@@ -477,7 +487,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:H29"/>
-  <sheetFormatPr defaultColWidth="8.72265625" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.73046875" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="9.13"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14.88"/>
@@ -636,83 +646,93 @@
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1"/>
-      <c r="B11" s="13"/>
-      <c r="C11" s="13"/>
-      <c r="D11" s="13"/>
-      <c r="E11" s="13"/>
-      <c r="F11" s="13"/>
+      <c r="B11" s="13" t="n">
+        <v>46289</v>
+      </c>
+      <c r="C11" s="14" t="s">
+        <v>6</v>
+      </c>
+      <c r="D11" s="14" t="s">
+        <v>7</v>
+      </c>
+      <c r="E11" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="F11" s="14" t="s">
+        <v>17</v>
+      </c>
       <c r="G11" s="1"/>
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1"/>
-      <c r="B12" s="14"/>
-      <c r="C12" s="14"/>
-      <c r="D12" s="14"/>
-      <c r="E12" s="14"/>
-      <c r="F12" s="14"/>
+      <c r="B12" s="15"/>
+      <c r="C12" s="15"/>
+      <c r="D12" s="15"/>
+      <c r="E12" s="15"/>
+      <c r="F12" s="15"/>
       <c r="G12" s="1"/>
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1"/>
-      <c r="B13" s="13"/>
-      <c r="C13" s="13"/>
-      <c r="D13" s="13"/>
-      <c r="E13" s="13"/>
-      <c r="F13" s="13"/>
+      <c r="B13" s="14"/>
+      <c r="C13" s="14"/>
+      <c r="D13" s="14"/>
+      <c r="E13" s="14"/>
+      <c r="F13" s="14"/>
       <c r="G13" s="1"/>
     </row>
     <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1"/>
-      <c r="B14" s="14"/>
-      <c r="C14" s="14"/>
-      <c r="D14" s="14"/>
-      <c r="E14" s="14"/>
-      <c r="F14" s="14"/>
+      <c r="B14" s="15"/>
+      <c r="C14" s="15"/>
+      <c r="D14" s="15"/>
+      <c r="E14" s="15"/>
+      <c r="F14" s="15"/>
       <c r="G14" s="1"/>
     </row>
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1"/>
-      <c r="B15" s="13"/>
-      <c r="C15" s="13"/>
-      <c r="D15" s="13"/>
-      <c r="E15" s="13"/>
-      <c r="F15" s="13"/>
+      <c r="B15" s="14"/>
+      <c r="C15" s="14"/>
+      <c r="D15" s="14"/>
+      <c r="E15" s="14"/>
+      <c r="F15" s="14"/>
       <c r="G15" s="1"/>
     </row>
     <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1"/>
-      <c r="B16" s="14"/>
-      <c r="C16" s="14"/>
-      <c r="D16" s="14"/>
-      <c r="E16" s="14"/>
-      <c r="F16" s="14"/>
+      <c r="B16" s="15"/>
+      <c r="C16" s="15"/>
+      <c r="D16" s="15"/>
+      <c r="E16" s="15"/>
+      <c r="F16" s="15"/>
       <c r="G16" s="1"/>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1"/>
-      <c r="B17" s="13"/>
-      <c r="C17" s="13"/>
-      <c r="D17" s="13"/>
-      <c r="E17" s="13"/>
-      <c r="F17" s="13"/>
+      <c r="B17" s="14"/>
+      <c r="C17" s="14"/>
+      <c r="D17" s="14"/>
+      <c r="E17" s="14"/>
+      <c r="F17" s="14"/>
       <c r="G17" s="1"/>
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1"/>
-      <c r="B18" s="14"/>
-      <c r="C18" s="14"/>
-      <c r="D18" s="14"/>
-      <c r="E18" s="14"/>
-      <c r="F18" s="14"/>
+      <c r="B18" s="15"/>
+      <c r="C18" s="15"/>
+      <c r="D18" s="15"/>
+      <c r="E18" s="15"/>
+      <c r="F18" s="15"/>
       <c r="G18" s="1"/>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1"/>
-      <c r="B19" s="13"/>
-      <c r="C19" s="13"/>
-      <c r="D19" s="13"/>
-      <c r="E19" s="13"/>
-      <c r="F19" s="13"/>
+      <c r="B19" s="14"/>
+      <c r="C19" s="14"/>
+      <c r="D19" s="14"/>
+      <c r="E19" s="14"/>
+      <c r="F19" s="14"/>
       <c r="G19" s="1"/>
     </row>
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -726,92 +746,92 @@
     </row>
     <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1"/>
-      <c r="B21" s="15" t="s">
-        <v>16</v>
-      </c>
-      <c r="C21" s="16"/>
-      <c r="D21" s="16"/>
-      <c r="E21" s="16"/>
-      <c r="F21" s="17"/>
+      <c r="B21" s="16" t="s">
+        <v>18</v>
+      </c>
+      <c r="C21" s="17"/>
+      <c r="D21" s="17"/>
+      <c r="E21" s="17"/>
+      <c r="F21" s="18"/>
       <c r="G21" s="1"/>
     </row>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1"/>
-      <c r="B22" s="18"/>
+      <c r="B22" s="19"/>
       <c r="C22" s="1" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="D22" s="1"/>
       <c r="E22" s="1"/>
-      <c r="F22" s="19"/>
+      <c r="F22" s="20"/>
       <c r="G22" s="1"/>
     </row>
     <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="1"/>
-      <c r="B23" s="18"/>
+      <c r="B23" s="19"/>
       <c r="C23" s="1" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="D23" s="1"/>
       <c r="E23" s="1"/>
-      <c r="F23" s="19"/>
+      <c r="F23" s="20"/>
       <c r="G23" s="1"/>
       <c r="H23" s="12"/>
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="1"/>
-      <c r="B24" s="18"/>
+      <c r="B24" s="19"/>
       <c r="C24" s="1" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D24" s="1"/>
       <c r="E24" s="1"/>
-      <c r="F24" s="19"/>
+      <c r="F24" s="20"/>
       <c r="G24" s="1"/>
       <c r="H24" s="12"/>
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="1"/>
-      <c r="B25" s="18"/>
+      <c r="B25" s="19"/>
       <c r="C25" s="1" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="D25" s="1"/>
       <c r="E25" s="1"/>
-      <c r="F25" s="19"/>
+      <c r="F25" s="20"/>
       <c r="G25" s="1"/>
     </row>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="1"/>
-      <c r="B26" s="18"/>
+      <c r="B26" s="19"/>
       <c r="C26" s="1" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D26" s="1"/>
       <c r="E26" s="1"/>
-      <c r="F26" s="19"/>
+      <c r="F26" s="20"/>
       <c r="G26" s="1"/>
     </row>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="1"/>
-      <c r="B27" s="18"/>
+      <c r="B27" s="19"/>
       <c r="C27" s="1" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D27" s="1"/>
       <c r="E27" s="1"/>
-      <c r="F27" s="19"/>
+      <c r="F27" s="20"/>
       <c r="G27" s="1"/>
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="1"/>
-      <c r="B28" s="20"/>
-      <c r="C28" s="21" t="s">
-        <v>23</v>
-      </c>
-      <c r="D28" s="21"/>
-      <c r="E28" s="21"/>
-      <c r="F28" s="22"/>
+      <c r="B28" s="21"/>
+      <c r="C28" s="22" t="s">
+        <v>25</v>
+      </c>
+      <c r="D28" s="22"/>
+      <c r="E28" s="22"/>
+      <c r="F28" s="23"/>
       <c r="G28" s="1"/>
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Ajout de la tâche dans la matrice des tâches
- Ajout de la tâche dans la matrice des tâches
</commit_message>
<xml_diff>
--- a/Matrice des tâches.xlsx
+++ b/Matrice des tâches.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="27">
   <si>
     <t xml:space="preserve">Matrice de répartition de charges (à remplir à chaque séance)</t>
   </si>
@@ -74,6 +74,9 @@
   </si>
   <si>
     <t xml:space="preserve">J’ai aussi bien réfléchit sur comment implémenter les collisions entre entité</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ajout des collisions entre entités </t>
   </si>
   <si>
     <t xml:space="preserve">Attention :</t>
@@ -312,7 +315,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -370,6 +373,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="2" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="3" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -487,7 +494,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:H29"/>
-  <sheetFormatPr defaultColWidth="8.73046875" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.7421875" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="9.13"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14.88"/>
@@ -665,11 +672,19 @@
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1"/>
-      <c r="B12" s="15"/>
-      <c r="C12" s="15"/>
-      <c r="D12" s="15"/>
-      <c r="E12" s="15"/>
-      <c r="F12" s="15"/>
+      <c r="B12" s="15" t="n">
+        <v>46290</v>
+      </c>
+      <c r="C12" s="16" t="s">
+        <v>6</v>
+      </c>
+      <c r="D12" s="16" t="s">
+        <v>7</v>
+      </c>
+      <c r="E12" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="F12" s="16"/>
       <c r="G12" s="1"/>
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -683,11 +698,11 @@
     </row>
     <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1"/>
-      <c r="B14" s="15"/>
-      <c r="C14" s="15"/>
-      <c r="D14" s="15"/>
-      <c r="E14" s="15"/>
-      <c r="F14" s="15"/>
+      <c r="B14" s="16"/>
+      <c r="C14" s="16"/>
+      <c r="D14" s="16"/>
+      <c r="E14" s="16"/>
+      <c r="F14" s="16"/>
       <c r="G14" s="1"/>
     </row>
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -701,11 +716,11 @@
     </row>
     <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1"/>
-      <c r="B16" s="15"/>
-      <c r="C16" s="15"/>
-      <c r="D16" s="15"/>
-      <c r="E16" s="15"/>
-      <c r="F16" s="15"/>
+      <c r="B16" s="16"/>
+      <c r="C16" s="16"/>
+      <c r="D16" s="16"/>
+      <c r="E16" s="16"/>
+      <c r="F16" s="16"/>
       <c r="G16" s="1"/>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -719,11 +734,11 @@
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1"/>
-      <c r="B18" s="15"/>
-      <c r="C18" s="15"/>
-      <c r="D18" s="15"/>
-      <c r="E18" s="15"/>
-      <c r="F18" s="15"/>
+      <c r="B18" s="16"/>
+      <c r="C18" s="16"/>
+      <c r="D18" s="16"/>
+      <c r="E18" s="16"/>
+      <c r="F18" s="16"/>
       <c r="G18" s="1"/>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -746,92 +761,92 @@
     </row>
     <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1"/>
-      <c r="B21" s="16" t="s">
-        <v>18</v>
-      </c>
-      <c r="C21" s="17"/>
-      <c r="D21" s="17"/>
-      <c r="E21" s="17"/>
-      <c r="F21" s="18"/>
+      <c r="B21" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="C21" s="18"/>
+      <c r="D21" s="18"/>
+      <c r="E21" s="18"/>
+      <c r="F21" s="19"/>
       <c r="G21" s="1"/>
     </row>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1"/>
-      <c r="B22" s="19"/>
+      <c r="B22" s="20"/>
       <c r="C22" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D22" s="1"/>
       <c r="E22" s="1"/>
-      <c r="F22" s="20"/>
+      <c r="F22" s="21"/>
       <c r="G22" s="1"/>
     </row>
     <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="1"/>
-      <c r="B23" s="19"/>
+      <c r="B23" s="20"/>
       <c r="C23" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D23" s="1"/>
       <c r="E23" s="1"/>
-      <c r="F23" s="20"/>
+      <c r="F23" s="21"/>
       <c r="G23" s="1"/>
       <c r="H23" s="12"/>
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="1"/>
-      <c r="B24" s="19"/>
+      <c r="B24" s="20"/>
       <c r="C24" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D24" s="1"/>
       <c r="E24" s="1"/>
-      <c r="F24" s="20"/>
+      <c r="F24" s="21"/>
       <c r="G24" s="1"/>
       <c r="H24" s="12"/>
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="1"/>
-      <c r="B25" s="19"/>
+      <c r="B25" s="20"/>
       <c r="C25" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D25" s="1"/>
       <c r="E25" s="1"/>
-      <c r="F25" s="20"/>
+      <c r="F25" s="21"/>
       <c r="G25" s="1"/>
     </row>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="1"/>
-      <c r="B26" s="19"/>
+      <c r="B26" s="20"/>
       <c r="C26" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D26" s="1"/>
       <c r="E26" s="1"/>
-      <c r="F26" s="20"/>
+      <c r="F26" s="21"/>
       <c r="G26" s="1"/>
     </row>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="1"/>
-      <c r="B27" s="19"/>
+      <c r="B27" s="20"/>
       <c r="C27" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D27" s="1"/>
       <c r="E27" s="1"/>
-      <c r="F27" s="20"/>
+      <c r="F27" s="21"/>
       <c r="G27" s="1"/>
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="1"/>
-      <c r="B28" s="21"/>
-      <c r="C28" s="22" t="s">
-        <v>25</v>
-      </c>
-      <c r="D28" s="22"/>
-      <c r="E28" s="22"/>
-      <c r="F28" s="23"/>
+      <c r="B28" s="22"/>
+      <c r="C28" s="23" t="s">
+        <v>26</v>
+      </c>
+      <c r="D28" s="23"/>
+      <c r="E28" s="23"/>
+      <c r="F28" s="24"/>
       <c r="G28" s="1"/>
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>